<commit_message>
Checkpoint: Se reemplazó el permiso de ingreso OAuth por autenticación interna. El sistema permanece cerrado mientras no exista ningún almacenero. El primer almacenero se registra con nombre, código y contraseña y recibe rol administrador; los siguientes ingresan con código y contraseña como operadores. Las contraseñas se guardan con hash scrypt, la sesión usa cookie JWT interna, se eliminó la redirección automática al portal externo, el formulario de alta de almaceneros solicita contraseña y la plantilla Excel incluye la columna contrasena. Se aplicó migración no destructiva y pasaron 6 pruebas automatizadas y el build de producción.
</commit_message>
<xml_diff>
--- a/plantilla_control_herramientas.xlsx
+++ b/plantilla_control_herramientas.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -472,10 +472,13 @@
       <c r="D1" t="str">
         <v>telefono</v>
       </c>
+      <c r="E1" t="str">
+        <v>contrasena</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>